<commit_message>
smaller rounds play at the same time
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -23000,89 +23000,89 @@
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="J2" s="37" t="inlineStr">
+      <c r="J2" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="K2" s="37" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="K2" s="38" t="inlineStr">
+      <c r="L2" s="38" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="L2" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
       <c r="M2" s="40" t="inlineStr">
         <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="N2" s="39" t="inlineStr">
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="N2" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="O2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P2" s="39" t="inlineStr">
         <is>
           <t>MD V - 2</t>
         </is>
       </c>
-      <c r="O2" s="37" t="inlineStr">
+      <c r="Q2" s="37" t="inlineStr">
         <is>
           <t>XD V - 2</t>
         </is>
       </c>
-      <c r="P2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q2" s="41" t="inlineStr">
+      <c r="R2" s="41" t="inlineStr">
         <is>
           <t>WD V - 1</t>
         </is>
       </c>
-      <c r="R2" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S2" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="T2" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="U2" s="37" t="inlineStr">
+      <c r="S2" s="37" t="inlineStr">
         <is>
           <t>XD V - 3</t>
         </is>
       </c>
-      <c r="V2" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
+      <c r="T2" s="39" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="U2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="V2" s="39" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
         </is>
       </c>
       <c r="W2" s="38" t="inlineStr">
         <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="X2" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="Y2" s="38" t="inlineStr">
-        <is>
           <t>MS V - 4</t>
         </is>
       </c>
-      <c r="Z2" s="37" t="inlineStr">
+      <c r="X2" s="37" t="inlineStr">
         <is>
           <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="Y2" s="36" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="Z2" s="49" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
         </is>
       </c>
     </row>
@@ -23127,84 +23127,89 @@
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="J3" s="37" t="inlineStr">
+      <c r="J3" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="K3" s="37" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="K3" s="38" t="inlineStr">
+      <c r="L3" s="38" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="L3" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
       <c r="M3" s="40" t="inlineStr">
         <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="N3" s="39" t="inlineStr">
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="N3" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="O3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P3" s="39" t="inlineStr">
         <is>
           <t>MD V - 2</t>
         </is>
       </c>
-      <c r="O3" s="37" t="inlineStr">
+      <c r="Q3" s="37" t="inlineStr">
         <is>
           <t>XD V - 2</t>
         </is>
       </c>
-      <c r="P3" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q3" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
       <c r="R3" s="41" t="inlineStr">
         <is>
           <t>WD V - 1</t>
         </is>
       </c>
-      <c r="S3" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="T3" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="U3" s="37" t="inlineStr">
+      <c r="S3" s="37" t="inlineStr">
         <is>
           <t>XD V - 3</t>
         </is>
       </c>
-      <c r="V3" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="W3" s="38" t="inlineStr">
+      <c r="T3" s="39" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="U3" s="38" t="inlineStr">
         <is>
           <t>MS V - 3</t>
         </is>
       </c>
-      <c r="X3" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="Y3" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
+      <c r="V3" s="41" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+      <c r="W3" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="X3" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="Y3" s="35" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="Z3" s="34" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
         </is>
       </c>
     </row>
@@ -23249,79 +23254,79 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J4" s="37" t="inlineStr">
+      <c r="J4" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="K4" s="37" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="K4" s="38" t="inlineStr">
+      <c r="L4" s="38" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="L4" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
       <c r="M4" s="40" t="inlineStr">
         <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="N4" s="39" t="inlineStr">
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="N4" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="O4" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P4" s="39" t="inlineStr">
         <is>
           <t>MD V - 2</t>
         </is>
       </c>
-      <c r="O4" s="37" t="inlineStr">
+      <c r="Q4" s="37" t="inlineStr">
         <is>
           <t>XD V - 2</t>
         </is>
       </c>
-      <c r="P4" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q4" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
       <c r="R4" s="41" t="inlineStr">
         <is>
           <t>WD V - 1</t>
         </is>
       </c>
-      <c r="S4" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="T4" s="36" t="inlineStr">
+      <c r="S4" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="T4" s="41" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="U4" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="V4" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="W4" s="36" t="inlineStr">
         <is>
           <t>XD A - 3</t>
         </is>
       </c>
-      <c r="U4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="V4" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="W4" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="X4" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
+      <c r="X4" s="44" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
         </is>
       </c>
     </row>
@@ -23366,79 +23371,79 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J5" s="37" t="inlineStr">
+      <c r="J5" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="K5" s="37" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="K5" s="38" t="inlineStr">
+      <c r="L5" s="38" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="L5" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="M5" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="N5" s="39" t="inlineStr">
+      <c r="M5" s="39" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="N5" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="O5" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="39" t="inlineStr">
         <is>
           <t>MD V - 2</t>
         </is>
       </c>
-      <c r="O5" s="37" t="inlineStr">
+      <c r="Q5" s="37" t="inlineStr">
         <is>
           <t>XD V - 2</t>
         </is>
       </c>
-      <c r="P5" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q5" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="R5" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="S5" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="T5" s="36" t="inlineStr">
+      <c r="R5" s="41" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="S5" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="T5" s="41" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="U5" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="V5" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="W5" s="36" t="inlineStr">
         <is>
           <t>XD A - 3</t>
         </is>
       </c>
-      <c r="U5" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="V5" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="W5" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="X5" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
+      <c r="X5" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
         </is>
       </c>
     </row>
@@ -23483,44 +23488,44 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J6" s="37" t="inlineStr">
+      <c r="J6" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="K6" s="37" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="K6" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
       <c r="L6" s="36" t="inlineStr">
         <is>
           <t>XD A - 2</t>
         </is>
       </c>
-      <c r="M6" s="33" t="inlineStr">
+      <c r="M6" s="39" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="N6" s="34" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="O6" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P6" s="33" t="inlineStr">
         <is>
           <t>MS A - 3</t>
         </is>
       </c>
-      <c r="N6" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="O6" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="P6" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="Q6" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
+      <c r="Q6" s="44" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
         </is>
       </c>
       <c r="R6" s="45" t="inlineStr">
@@ -23528,14 +23533,14 @@
           <t>MS C - 3</t>
         </is>
       </c>
-      <c r="S6" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="T6" s="48" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
+      <c r="S6" s="49" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="T6" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
         </is>
       </c>
       <c r="U6" s="49" t="inlineStr">
@@ -23543,19 +23548,19 @@
           <t>WD A - 2</t>
         </is>
       </c>
-      <c r="V6" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="W6" s="49" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="X6" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
+      <c r="V6" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="W6" s="35" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="X6" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
         </is>
       </c>
     </row>
@@ -23600,59 +23605,59 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J7" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="K7" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="L7" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="M7" s="33" t="inlineStr">
+      <c r="J7" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="K7" s="35" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="L7" s="36" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="M7" s="44" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="N7" s="34" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="O7" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P7" s="33" t="inlineStr">
         <is>
           <t>MS A - 3</t>
         </is>
       </c>
-      <c r="N7" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="O7" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="P7" s="49" t="inlineStr">
+      <c r="Q7" s="44" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="R7" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="S7" s="49" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="Q7" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="R7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="S7" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="T7" s="48" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
+      <c r="T7" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
         </is>
       </c>
       <c r="U7" s="49" t="inlineStr">
@@ -23660,19 +23665,14 @@
           <t>WD A - 2</t>
         </is>
       </c>
-      <c r="V7" s="35" t="inlineStr">
+      <c r="V7" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="W7" s="35" t="inlineStr">
         <is>
           <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="W7" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="X7" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
         </is>
       </c>
     </row>
@@ -23717,59 +23717,59 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J8" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="K8" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="L8" s="34" t="inlineStr">
+      <c r="J8" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="K8" s="35" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="L8" s="36" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="M8" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="N8" s="34" t="inlineStr">
         <is>
           <t>MD B - 3</t>
         </is>
       </c>
-      <c r="M8" s="33" t="inlineStr">
+      <c r="O8" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P8" s="33" t="inlineStr">
         <is>
           <t>MS A - 3</t>
         </is>
       </c>
-      <c r="N8" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="O8" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="P8" s="49" t="inlineStr">
+      <c r="Q8" s="51" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="R8" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="S8" s="49" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="Q8" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="R8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="S8" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="T8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
+      <c r="T8" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
         </is>
       </c>
       <c r="U8" s="34" t="inlineStr">
@@ -23777,19 +23777,14 @@
           <t>MD B - 4</t>
         </is>
       </c>
-      <c r="V8" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="W8" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
-        </is>
-      </c>
-      <c r="X8" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
+      <c r="V8" s="43" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="W8" s="48" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
         </is>
       </c>
     </row>
@@ -23834,44 +23829,44 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J9" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="K9" s="36" t="inlineStr">
+      <c r="J9" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="K9" s="35" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="L9" s="36" t="inlineStr">
         <is>
           <t>XD A - 2</t>
         </is>
       </c>
-      <c r="L9" s="34" t="inlineStr">
+      <c r="M9" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="N9" s="34" t="inlineStr">
         <is>
           <t>MD B - 3</t>
         </is>
       </c>
-      <c r="M9" s="33" t="inlineStr">
+      <c r="O9" s="40" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P9" s="33" t="inlineStr">
         <is>
           <t>MS A - 3</t>
         </is>
       </c>
-      <c r="N9" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="O9" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="P9" s="49" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Q9" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
+      <c r="Q9" s="51" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
         </is>
       </c>
       <c r="R9" s="45" t="inlineStr">
@@ -23879,9 +23874,9 @@
           <t>MS C - 3</t>
         </is>
       </c>
-      <c r="S9" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
+      <c r="S9" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
         </is>
       </c>
       <c r="T9" s="45" t="inlineStr">
@@ -23894,9 +23889,9 @@
           <t>MD B - 4</t>
         </is>
       </c>
-      <c r="V9" s="48" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
+      <c r="V9" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
         </is>
       </c>
       <c r="W9" s="51" t="inlineStr">
@@ -23946,69 +23941,69 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J10" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="K10" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="L10" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="M10" s="35" t="inlineStr">
+      <c r="J10" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="K10" s="35" t="inlineStr">
         <is>
           <t>MS B - 3</t>
         </is>
       </c>
-      <c r="N10" s="50" t="inlineStr">
+      <c r="L10" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="M10" s="50" t="inlineStr">
         <is>
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="O10" s="51" t="inlineStr">
+      <c r="N10" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="O10" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="P10" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="Q10" s="51" t="inlineStr">
         <is>
           <t>XD C - 1</t>
         </is>
       </c>
-      <c r="P10" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Q10" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="S10" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="T10" s="52" t="inlineStr">
-        <is>
           <t>WD C - 2</t>
         </is>
       </c>
-      <c r="U10" s="51" t="inlineStr">
+      <c r="S10" s="51" t="inlineStr">
         <is>
           <t>XD C - 2</t>
         </is>
       </c>
-      <c r="V10" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
+      <c r="T10" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="U10" s="48" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="V10" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
         </is>
       </c>
     </row>
@@ -24053,59 +24048,64 @@
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J11" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="K11" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="M11" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="N11" s="50" t="inlineStr">
+      <c r="J11" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="K11" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="L11" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="M11" s="50" t="inlineStr">
         <is>
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="O11" s="51" t="inlineStr">
+      <c r="N11" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="O11" s="50" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="P11" s="47" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="Q11" s="51" t="inlineStr">
         <is>
           <t>XD C - 1</t>
         </is>
       </c>
-      <c r="P11" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Q11" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>WD C - 1</t>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="S11" s="51" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
         </is>
       </c>
       <c r="T11" s="52" t="inlineStr">
         <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="U11" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="V11" s="52" t="inlineStr">
-        <is>
           <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="U11" s="48" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed print to excel, weak collisions added
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Entries HBC Premier Elite 2024" sheetId="1" state="visible" r:id="rId1"/>
@@ -75,14 +75,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF8E1"/>
         <bgColor rgb="FFFFF8E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
-        <bgColor rgb="FFE8F5E9"/>
+        <fgColor rgb="FFF48FB1"/>
+        <bgColor rgb="FFF48FB1"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,20 +99,62 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFDE0E0"/>
+        <bgColor rgb="FFFDE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEC407A"/>
+        <bgColor rgb="FFEC407A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF66BB6A"/>
+        <bgColor rgb="FF66BB6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF42A5F5"/>
+        <bgColor rgb="FF42A5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFECB3"/>
+        <bgColor rgb="FFFFECB3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3F2FD"/>
+        <bgColor rgb="FFE3F2FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBBDEFB"/>
+        <bgColor rgb="FFBBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90CAF9"/>
+        <bgColor rgb="FF90CAF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF8BBD0"/>
         <bgColor rgb="FFF8BBD0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF48FB1"/>
-        <bgColor rgb="FFF48FB1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFDE0E0"/>
-        <bgColor rgb="FFFDE0E0"/>
+        <fgColor rgb="FFFFCA28"/>
+        <bgColor rgb="FFFFCA28"/>
       </patternFill>
     </fill>
     <fill>
@@ -117,50 +165,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF66BB6A"/>
-        <bgColor rgb="FF66BB6A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCA28"/>
-        <bgColor rgb="FFFFCA28"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEC407A"/>
-        <bgColor rgb="FFEC407A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE3F2FD"/>
-        <bgColor rgb="FFE3F2FD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF42A5F5"/>
-        <bgColor rgb="FF42A5F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBBDEFB"/>
-        <bgColor rgb="FFBBDEFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFECB3"/>
-        <bgColor rgb="FFFFECB3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF90CAF9"/>
-        <bgColor rgb="FF90CAF9"/>
+        <fgColor rgb="FF81C784"/>
+        <bgColor rgb="FF81C784"/>
       </patternFill>
     </fill>
     <fill>
@@ -171,20 +177,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF81C784"/>
-        <bgColor rgb="FF81C784"/>
+        <fgColor rgb="FFC8E6C9"/>
+        <bgColor rgb="FFC8E6C9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFD54F"/>
         <bgColor rgb="FFFFD54F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC8E6C9"/>
-        <bgColor rgb="FFC8E6C9"/>
       </patternFill>
     </fill>
     <fill>
@@ -207,32 +207,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F48FB1"/>
-        <bgColor rgb="00F48FB1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE082"/>
-        <bgColor rgb="00FFE082"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDE0E0"/>
-        <bgColor rgb="00FDE0E0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EC407A"/>
-        <bgColor rgb="00EC407A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0066BB6A"/>
-        <bgColor rgb="0066BB6A"/>
+        <fgColor rgb="00FFECB3"/>
+        <bgColor rgb="00FFECB3"/>
       </patternFill>
     </fill>
     <fill>
@@ -243,8 +219,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFECB3"/>
-        <bgColor rgb="00FFECB3"/>
+        <fgColor rgb="00F8BBD0"/>
+        <bgColor rgb="00F8BBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F48FB1"/>
+        <bgColor rgb="00F48FB1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCA28"/>
+        <bgColor rgb="00FFCA28"/>
       </patternFill>
     </fill>
     <fill>
@@ -261,20 +249,50 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FDE0E0"/>
+        <bgColor rgb="00FDE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="0090CAF9"/>
         <bgColor rgb="0090CAF9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8BBD0"/>
-        <bgColor rgb="00F8BBD0"/>
+        <fgColor rgb="00FFD54F"/>
+        <bgColor rgb="00FFD54F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCA28"/>
-        <bgColor rgb="00FFCA28"/>
+        <fgColor rgb="0066BB6A"/>
+        <bgColor rgb="0066BB6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE082"/>
+        <bgColor rgb="00FFE082"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EC407A"/>
+        <bgColor rgb="00EC407A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0064B5F6"/>
+        <bgColor rgb="0064B5F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F06292"/>
+        <bgColor rgb="00F06292"/>
       </patternFill>
     </fill>
     <fill>
@@ -291,26 +309,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0064B5F6"/>
-        <bgColor rgb="0064B5F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C8E6C9"/>
         <bgColor rgb="00C8E6C9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD54F"/>
-        <bgColor rgb="00FFD54F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F06292"/>
-        <bgColor rgb="00F06292"/>
       </patternFill>
     </fill>
   </fills>
@@ -364,45 +364,45 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18281,14 +18281,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C283"/>
+  <dimension ref="A1:C254"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="29.6640625" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="20.6640625" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
     <col width="34.33203125" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
-    <col width="8.83203125" customWidth="1" style="7" min="4" max="10"/>
-    <col width="8.83203125" customWidth="1" style="7" min="11" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="7" min="4" max="11"/>
+    <col width="8.83203125" customWidth="1" style="7" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" thickBot="1">
@@ -20162,7 +20162,6 @@
           <t>MD B, MD C</t>
         </is>
       </c>
-      <c r="C151" s="7" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -21429,122 +21428,6 @@
           <t>WD V, WS V</t>
         </is>
       </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="7" t="n"/>
-      <c r="B255" s="7" t="n"/>
-    </row>
-    <row r="256">
-      <c r="A256" s="7" t="n"/>
-      <c r="B256" s="7" t="n"/>
-    </row>
-    <row r="257">
-      <c r="A257" s="7" t="n"/>
-      <c r="B257" s="7" t="n"/>
-    </row>
-    <row r="258">
-      <c r="A258" s="7" t="n"/>
-      <c r="B258" s="7" t="n"/>
-    </row>
-    <row r="259">
-      <c r="A259" s="7" t="n"/>
-      <c r="B259" s="7" t="n"/>
-    </row>
-    <row r="260">
-      <c r="A260" s="7" t="n"/>
-      <c r="B260" s="7" t="n"/>
-    </row>
-    <row r="261">
-      <c r="A261" s="7" t="n"/>
-      <c r="B261" s="7" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="7" t="n"/>
-      <c r="B262" s="7" t="n"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="7" t="n"/>
-      <c r="B263" s="7" t="n"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="7" t="n"/>
-      <c r="B264" s="7" t="n"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="7" t="n"/>
-      <c r="B265" s="7" t="n"/>
-    </row>
-    <row r="266">
-      <c r="A266" s="7" t="n"/>
-      <c r="B266" s="7" t="n"/>
-    </row>
-    <row r="267">
-      <c r="A267" s="7" t="n"/>
-      <c r="B267" s="7" t="n"/>
-    </row>
-    <row r="268">
-      <c r="A268" s="7" t="n"/>
-      <c r="B268" s="7" t="n"/>
-    </row>
-    <row r="269">
-      <c r="A269" s="7" t="n"/>
-      <c r="B269" s="7" t="n"/>
-    </row>
-    <row r="270">
-      <c r="A270" s="7" t="n"/>
-      <c r="B270" s="7" t="n"/>
-    </row>
-    <row r="271">
-      <c r="A271" s="7" t="n"/>
-      <c r="B271" s="7" t="n"/>
-    </row>
-    <row r="272">
-      <c r="A272" s="7" t="n"/>
-      <c r="B272" s="7" t="n"/>
-    </row>
-    <row r="273">
-      <c r="A273" s="7" t="n"/>
-      <c r="B273" s="7" t="n"/>
-    </row>
-    <row r="274">
-      <c r="A274" s="7" t="n"/>
-      <c r="B274" s="7" t="n"/>
-    </row>
-    <row r="275">
-      <c r="A275" s="7" t="n"/>
-      <c r="B275" s="7" t="n"/>
-    </row>
-    <row r="276">
-      <c r="A276" s="7" t="n"/>
-      <c r="B276" s="7" t="n"/>
-    </row>
-    <row r="277">
-      <c r="A277" s="7" t="n"/>
-      <c r="B277" s="7" t="n"/>
-    </row>
-    <row r="278">
-      <c r="A278" s="7" t="n"/>
-      <c r="B278" s="7" t="n"/>
-    </row>
-    <row r="279">
-      <c r="A279" s="7" t="n"/>
-      <c r="B279" s="7" t="n"/>
-    </row>
-    <row r="280">
-      <c r="A280" s="7" t="n"/>
-      <c r="B280" s="7" t="n"/>
-    </row>
-    <row r="281">
-      <c r="A281" s="7" t="n"/>
-      <c r="B281" s="7" t="n"/>
-    </row>
-    <row r="282">
-      <c r="A282" s="7" t="n"/>
-      <c r="B282" s="7" t="n"/>
-    </row>
-    <row r="283">
-      <c r="A283" s="7" t="n"/>
-      <c r="B283" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22956,7 +22839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Z11"/>
+  <dimension ref="B2:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -22972,7 +22855,7 @@
       </c>
       <c r="D2" s="34" t="inlineStr">
         <is>
-          <t>MD B - 1</t>
+          <t>XD V - 1</t>
         </is>
       </c>
       <c r="E2" s="33" t="inlineStr">
@@ -22980,107 +22863,132 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F2" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="G2" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
+      <c r="F2" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G2" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
         </is>
       </c>
       <c r="H2" s="36" t="inlineStr">
         <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="I2" s="37" t="inlineStr">
+        <is>
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="I2" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J2" s="43" t="inlineStr">
+      <c r="J2" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="K2" s="36" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L2" s="39" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M2" s="34" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N2" s="39" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="K2" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="L2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="M2" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="N2" s="47" t="inlineStr">
+      <c r="O2" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P2" s="40" t="inlineStr">
         <is>
           <t>WS B - 2</t>
         </is>
       </c>
-      <c r="O2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P2" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
       <c r="Q2" s="37" t="inlineStr">
         <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="R2" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S2" s="37" t="inlineStr">
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="R2" s="36" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="S2" s="41" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="T2" s="34" t="inlineStr">
         <is>
           <t>XD V - 3</t>
         </is>
       </c>
-      <c r="T2" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="U2" s="38" t="inlineStr">
+      <c r="U2" s="41" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="V2" s="35" t="inlineStr">
         <is>
           <t>MS V - 3</t>
         </is>
       </c>
-      <c r="V2" s="39" t="inlineStr">
+      <c r="W2" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="X2" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+      <c r="Y2" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="Z2" s="34" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AA2" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AB2" s="36" t="inlineStr">
         <is>
           <t>MD V - 4</t>
         </is>
       </c>
-      <c r="W2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="X2" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="Y2" s="36" t="inlineStr">
+      <c r="AC2" s="37" t="inlineStr">
         <is>
           <t>XD A - 4</t>
         </is>
       </c>
-      <c r="Z2" s="49" t="inlineStr">
+      <c r="AD2" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AE2" s="44" t="inlineStr">
         <is>
           <t>WD A - 3</t>
         </is>
@@ -23092,14 +23000,14 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C3" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
+      <c r="C3" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
         </is>
       </c>
       <c r="D3" s="34" t="inlineStr">
         <is>
-          <t>MD B - 1</t>
+          <t>XD V - 1</t>
         </is>
       </c>
       <c r="E3" s="33" t="inlineStr">
@@ -23107,109 +23015,114 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F3" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="G3" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G3" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
         </is>
       </c>
       <c r="H3" s="36" t="inlineStr">
         <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="I3" s="37" t="inlineStr">
+        <is>
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="I3" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J3" s="43" t="inlineStr">
+      <c r="J3" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="K3" s="36" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L3" s="39" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M3" s="34" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N3" s="39" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="K3" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="L3" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="M3" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="N3" s="47" t="inlineStr">
+      <c r="O3" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P3" s="40" t="inlineStr">
         <is>
           <t>WS B - 2</t>
         </is>
       </c>
-      <c r="O3" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P3" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
       <c r="Q3" s="37" t="inlineStr">
         <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="R3" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S3" s="37" t="inlineStr">
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="R3" s="36" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="S3" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="T3" s="34" t="inlineStr">
         <is>
           <t>XD V - 3</t>
         </is>
       </c>
-      <c r="T3" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="U3" s="38" t="inlineStr">
+      <c r="U3" s="41" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="V3" s="35" t="inlineStr">
         <is>
           <t>MS V - 3</t>
         </is>
       </c>
-      <c r="V3" s="41" t="inlineStr">
+      <c r="W3" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="X3" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="Y3" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="Z3" s="40" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AB3" s="46" t="inlineStr">
         <is>
           <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="W3" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="X3" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="Y3" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="Z3" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
         </is>
       </c>
     </row>
@@ -23219,14 +23132,14 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
+      <c r="C4" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
         </is>
       </c>
       <c r="D4" s="34" t="inlineStr">
         <is>
-          <t>MD B - 1</t>
+          <t>XD V - 1</t>
         </is>
       </c>
       <c r="E4" s="33" t="inlineStr">
@@ -23234,99 +23147,114 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F4" s="43" t="inlineStr">
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G4" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="H4" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J4" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="K4" s="36" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L4" s="39" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G4" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="H4" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I4" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="J4" s="43" t="inlineStr">
+      <c r="M4" s="34" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N4" s="39" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="K4" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="L4" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="M4" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="N4" s="47" t="inlineStr">
+      <c r="O4" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P4" s="40" t="inlineStr">
         <is>
           <t>WS B - 2</t>
         </is>
       </c>
-      <c r="O4" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P4" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="Q4" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="R4" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="T4" s="41" t="inlineStr">
+      <c r="Q4" s="47" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="R4" s="46" t="inlineStr">
         <is>
           <t>WD V - 2</t>
         </is>
       </c>
-      <c r="U4" s="40" t="inlineStr">
+      <c r="S4" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="T4" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="U4" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="V4" s="38" t="inlineStr">
         <is>
           <t>WS V - 3</t>
         </is>
       </c>
-      <c r="V4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="W4" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="X4" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
+      <c r="W4" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="X4" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="Y4" s="42" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="Z4" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
+        </is>
+      </c>
+      <c r="AB4" s="39" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
         </is>
       </c>
     </row>
@@ -23343,7 +23271,7 @@
       </c>
       <c r="D5" s="34" t="inlineStr">
         <is>
-          <t>MD B - 1</t>
+          <t>XD V - 1</t>
         </is>
       </c>
       <c r="E5" s="33" t="inlineStr">
@@ -23351,99 +23279,99 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F5" s="43" t="inlineStr">
+      <c r="F5" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="H5" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I5" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J5" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="K5" s="36" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L5" s="39" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G5" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="H5" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I5" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="J5" s="43" t="inlineStr">
+      <c r="M5" s="34" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N5" s="39" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="K5" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="L5" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="M5" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="N5" s="47" t="inlineStr">
+      <c r="O5" s="35" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="40" t="inlineStr">
         <is>
           <t>WS B - 2</t>
         </is>
       </c>
-      <c r="O5" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P5" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="Q5" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="R5" s="41" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S5" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="T5" s="41" t="inlineStr">
+      <c r="R5" s="46" t="inlineStr">
         <is>
           <t>WD V - 2</t>
         </is>
       </c>
-      <c r="U5" s="40" t="inlineStr">
+      <c r="S5" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="T5" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="U5" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="V5" s="38" t="inlineStr">
         <is>
           <t>WS V - 3</t>
         </is>
       </c>
-      <c r="V5" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="W5" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="X5" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
+      <c r="W5" s="41" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="X5" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="Y5" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
         </is>
       </c>
     </row>
@@ -23458,9 +23386,9 @@
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="D6" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
         </is>
       </c>
       <c r="E6" s="33" t="inlineStr">
@@ -23468,97 +23396,92 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F6" s="43" t="inlineStr">
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="G6" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H6" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I6" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J6" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K6" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="L6" s="39" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G6" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="H6" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I6" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="J6" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="K6" s="37" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="L6" s="36" t="inlineStr">
+      <c r="M6" s="37" t="inlineStr">
         <is>
           <t>XD A - 2</t>
         </is>
       </c>
-      <c r="M6" s="39" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="N6" s="34" t="inlineStr">
+      <c r="O6" s="46" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="P6" s="48" t="inlineStr">
         <is>
           <t>MD B - 3</t>
         </is>
       </c>
-      <c r="O6" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="P6" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="Q6" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="R6" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
+      <c r="R6" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
         </is>
       </c>
       <c r="S6" s="49" t="inlineStr">
         <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="T6" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="U6" s="49" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="V6" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="W6" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="X6" s="46" t="inlineStr">
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="T6" s="40" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="U6" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="V6" s="39" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="W6" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="X6" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="Y6" s="51" t="inlineStr">
         <is>
           <t>MD C - 4</t>
         </is>
@@ -23575,9 +23498,9 @@
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="D7" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
@@ -23585,94 +23508,84 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F7" s="43" t="inlineStr">
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="G7" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H7" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I7" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J7" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K7" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="L7" s="39" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G7" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="H7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I7" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="J7" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="K7" s="35" t="inlineStr">
+      <c r="M7" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="O7" s="46" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="P7" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="R7" s="43" t="inlineStr">
         <is>
           <t>MS B - 3</t>
         </is>
       </c>
-      <c r="L7" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="M7" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="N7" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O7" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="P7" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="Q7" s="44" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="R7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
       <c r="S7" s="49" t="inlineStr">
         <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="T7" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="U7" s="49" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="V7" s="43" t="inlineStr">
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="T7" s="40" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="U7" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="V7" s="39" t="inlineStr">
         <is>
           <t>XD B - 3</t>
         </is>
       </c>
-      <c r="W7" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
+      <c r="W7" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
         </is>
       </c>
     </row>
@@ -23687,104 +23600,79 @@
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="D8" s="46" t="inlineStr">
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="G8" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H8" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I8" s="51" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="E8" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="F8" s="43" t="inlineStr">
+      <c r="J8" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K8" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="L8" s="39" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G8" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="H8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I8" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="J8" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="K8" s="35" t="inlineStr">
+      <c r="M8" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="O8" s="46" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="P8" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="R8" s="43" t="inlineStr">
         <is>
           <t>MS B - 3</t>
         </is>
       </c>
-      <c r="L8" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="M8" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="N8" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O8" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="P8" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="Q8" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="R8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="S8" s="49" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="T8" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="U8" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="V8" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="W8" s="48" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
+      <c r="S8" s="51" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="U8" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
         </is>
       </c>
     </row>
@@ -23799,104 +23687,79 @@
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="D9" s="46" t="inlineStr">
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G9" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H9" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I9" s="51" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="E9" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="F9" s="43" t="inlineStr">
+      <c r="J9" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K9" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="L9" s="39" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I9" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="J9" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="K9" s="35" t="inlineStr">
+      <c r="M9" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="O9" s="46" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="P9" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="R9" s="43" t="inlineStr">
         <is>
           <t>MS B - 3</t>
         </is>
       </c>
-      <c r="L9" s="36" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="M9" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="N9" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O9" s="40" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="P9" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="Q9" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="R9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="S9" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="T9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="U9" s="34" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="V9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="W9" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
+      <c r="S9" s="51" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="U9" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
         </is>
       </c>
     </row>
@@ -23906,104 +23769,64 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D10" s="46" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G10" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H10" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I10" s="51" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="E10" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="F10" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="G10" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H10" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I10" s="34" t="inlineStr">
+      <c r="J10" s="48" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J10" s="46" t="inlineStr">
+      <c r="K10" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="M10" s="51" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="K10" s="35" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="L10" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="M10" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="N10" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="O10" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="P10" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="Q10" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="R10" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="S10" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="T10" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="U10" s="48" t="inlineStr">
+      <c r="O10" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="R10" s="50" t="inlineStr">
         <is>
           <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="V10" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
         </is>
       </c>
     </row>
@@ -24013,99 +23836,163 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C11" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D11" s="46" t="inlineStr">
+      <c r="C11" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G11" s="45" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H11" s="43" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="I11" s="51" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="J11" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K11" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="M11" s="51" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="O11" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="R11" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E12" s="47" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="F12" s="43" t="inlineStr">
         <is>
           <t>MS B - 1</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="G11" s="45" t="inlineStr">
+      <c r="G12" s="45" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="H11" s="45" t="inlineStr">
+      <c r="H12" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="I12" s="51" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J12" s="48" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K12" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="M12" s="51" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="O12" s="47" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E13" s="47" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="G13" s="45" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="I11" s="34" t="inlineStr">
+      <c r="H13" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="I13" s="51" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J13" s="48" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="J11" s="46" t="inlineStr">
+      <c r="K13" s="49" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="M13" s="51" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="K11" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="L11" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="M11" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="N11" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="O11" s="50" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="P11" s="47" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="Q11" s="51" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="R11" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="S11" s="51" t="inlineStr">
+      <c r="O13" s="47" t="inlineStr">
         <is>
           <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="T11" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-      <c r="U11" s="48" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
blocks all rounds from beeing split between saturday and sunday
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Entries HBC Premier Elite 2024" sheetId="1" state="visible" r:id="rId1"/>
@@ -60,7 +60,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="43">
+  <fills count="44">
     <fill>
       <patternFill/>
     </fill>
@@ -87,32 +87,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF48FB1"/>
-        <bgColor rgb="FFF48FB1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE082"/>
-        <bgColor rgb="FFFFE082"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFDE0E0"/>
-        <bgColor rgb="FFFDE0E0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEC407A"/>
-        <bgColor rgb="FFEC407A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF66BB6A"/>
-        <bgColor rgb="FF66BB6A"/>
+        <fgColor rgb="FFFFECB3"/>
+        <bgColor rgb="FFFFECB3"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,8 +99,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFECB3"/>
-        <bgColor rgb="FFFFECB3"/>
+        <fgColor rgb="FFF8BBD0"/>
+        <bgColor rgb="FFF8BBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF48FB1"/>
+        <bgColor rgb="FFF48FB1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCA28"/>
+        <bgColor rgb="FFFFCA28"/>
       </patternFill>
     </fill>
     <fill>
@@ -141,20 +129,50 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFDE0E0"/>
+        <bgColor rgb="FFFDE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF90CAF9"/>
         <bgColor rgb="FF90CAF9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8BBD0"/>
-        <bgColor rgb="FFF8BBD0"/>
+        <fgColor rgb="FFFFD54F"/>
+        <bgColor rgb="FFFFD54F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCA28"/>
-        <bgColor rgb="FFFFCA28"/>
+        <fgColor rgb="FF66BB6A"/>
+        <bgColor rgb="FF66BB6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE082"/>
+        <bgColor rgb="FFFFE082"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEC407A"/>
+        <bgColor rgb="FFEC407A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF64B5F6"/>
+        <bgColor rgb="FF64B5F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF06292"/>
+        <bgColor rgb="FFF06292"/>
       </patternFill>
     </fill>
     <fill>
@@ -171,26 +189,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF64B5F6"/>
-        <bgColor rgb="FF64B5F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC8E6C9"/>
         <bgColor rgb="FFC8E6C9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFD54F"/>
-        <bgColor rgb="FFFFD54F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF06292"/>
-        <bgColor rgb="FFF06292"/>
+        <fgColor theme="9" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -261,12 +267,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD54F"/>
-        <bgColor rgb="00FFD54F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0066BB6A"/>
         <bgColor rgb="0066BB6A"/>
       </patternFill>
@@ -279,20 +279,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="0064B5F6"/>
+        <bgColor rgb="0064B5F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EC407A"/>
         <bgColor rgb="00EC407A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0064B5F6"/>
-        <bgColor rgb="0064B5F6"/>
+        <fgColor rgb="00FFD54F"/>
+        <bgColor rgb="00FFD54F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F06292"/>
-        <bgColor rgb="00F06292"/>
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
     <fill>
@@ -309,8 +315,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
-        <bgColor rgb="00C8E6C9"/>
+        <fgColor rgb="00F06292"/>
+        <bgColor rgb="00F06292"/>
       </patternFill>
     </fill>
   </fills>
@@ -335,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -364,45 +370,46 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="43" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11981,7 +11988,9 @@
   <dimension ref="A2:BB138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
-    <col width="11" customWidth="1" style="2" min="1" max="59"/>
+    <col width="11" customWidth="1" style="2" min="1" max="43"/>
+    <col width="32.5" customWidth="1" style="2" min="44" max="44"/>
+    <col width="11" customWidth="1" style="2" min="45" max="59"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -14055,7 +14064,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="AO25" s="2" t="inlineStr">
+      <c r="AO25" s="33" t="inlineStr">
         <is>
           <t>En klass måste ha min 60 min mällan sina rundor</t>
         </is>
@@ -14079,7 +14088,7 @@
           <t>XD B</t>
         </is>
       </c>
-      <c r="AO26" s="2" t="inlineStr">
+      <c r="AO26" s="33" t="inlineStr">
         <is>
           <t>Alla matcher i en runda måste sättas in i max två efterföljande (jämna) tidsslots</t>
         </is>
@@ -14109,7 +14118,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="AO28" s="2" t="inlineStr">
+      <c r="AO28" s="33" t="inlineStr">
         <is>
           <t>En tidsslot kan ha max 10 matcher</t>
         </is>
@@ -14715,7 +14724,7 @@
           <t>MD B</t>
         </is>
       </c>
-      <c r="AO32" s="2" t="inlineStr">
+      <c r="AO32" s="33" t="inlineStr">
         <is>
           <t>Innom en nivå måste alla rundor i kolliderande klasser spelas med minst 1 tom tidsslots mällanrum</t>
         </is>
@@ -14870,7 +14879,7 @@
           <t>MD B</t>
         </is>
       </c>
-      <c r="AO33" s="2" t="inlineStr">
+      <c r="AO33" s="33" t="inlineStr">
         <is>
           <t>Rundor i kolliderande klasser som inte hör till samma nivå får inte spelas på samma tidsslot</t>
         </is>
@@ -15155,7 +15164,7 @@
           <t>MD A</t>
         </is>
       </c>
-      <c r="AO35" s="2" t="inlineStr">
+      <c r="AO35" s="33" t="inlineStr">
         <is>
           <t>Alla matcher ska spelas exakt en gång</t>
         </is>
@@ -15285,7 +15294,7 @@
           <t>MD A</t>
         </is>
       </c>
-      <c r="AO36" s="2" t="inlineStr">
+      <c r="AO36" s="33" t="inlineStr">
         <is>
           <t>Alla icke domarmatcher får bara spelas i timeslots som är prick och halv</t>
         </is>
@@ -18287,8 +18296,8 @@
     <col width="29.6640625" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="20.6640625" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
     <col width="34.33203125" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
-    <col width="8.83203125" customWidth="1" style="7" min="4" max="11"/>
-    <col width="8.83203125" customWidth="1" style="7" min="12" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="7" min="4" max="12"/>
+    <col width="8.83203125" customWidth="1" style="7" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" thickBot="1">
@@ -22839,1160 +22848,1160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AE13"/>
+  <dimension ref="B2:AM13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="33" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C2" s="33" t="inlineStr">
+      <c r="C2" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="D2" s="34" t="inlineStr">
+      <c r="D2" s="35" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="E2" s="33" t="inlineStr">
+      <c r="E2" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F2" s="35" t="inlineStr">
+      <c r="F2" s="36" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="G2" s="33" t="inlineStr">
+      <c r="G2" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="I2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="O2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="P2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="Q2" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="R2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="S2" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="AA2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AB2" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AC2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AD2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AE2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AF2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AG2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AH2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AI2" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AJ2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+      <c r="AK2" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AL2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="AM2" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="E3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G3" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="I3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J3" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L3" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="O3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="P3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="Q3" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="R3" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="S3" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="AA3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AB3" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AC3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AD3" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AE3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AF3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AG3" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="AH3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
+        </is>
+      </c>
+      <c r="AI3" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AJ3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="AK3" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AL3" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F4" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G4" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J4" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K4" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L4" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M4" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="O4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="P4" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="Q4" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="R4" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="S4" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="AA4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AB4" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AC4" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AD4" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AE4" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AF4" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AG4" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="AH4" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AI4" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AJ4" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AK4" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="AL4" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F5" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="G5" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I5" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K5" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="L5" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M5" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="N5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="O5" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="Q5" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="R5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AA5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AB5" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AC5" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AE5" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AF5" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AI5" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AJ5" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="E6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F6" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="G6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H6" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I6" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J6" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M6" s="34" t="inlineStr">
         <is>
           <t>MS A - 3</t>
         </is>
       </c>
-      <c r="H2" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="I2" s="37" t="inlineStr">
+      <c r="N6" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="P6" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AA6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AB6" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AC6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AE6" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AF6" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AI6" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D7" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F7" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="G7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H7" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I7" s="39" t="inlineStr">
         <is>
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="J2" s="38" t="inlineStr">
+      <c r="J7" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K7" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="L7" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="N7" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="P7" s="47" t="inlineStr">
         <is>
           <t>WS V - 2</t>
         </is>
       </c>
-      <c r="K2" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L2" s="39" t="inlineStr">
+      <c r="AA7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AB7" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AC7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AE7" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AF7" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AI7" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F8" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H8" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I8" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J8" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K8" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="L8" s="41" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="M2" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N2" s="39" t="inlineStr">
+      <c r="M8" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="P8" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AA8" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AC8" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+      <c r="AF8" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E9" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F9" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H9" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I9" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J9" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="K9" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="L9" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M9" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="P9" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AA9" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C10" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E10" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="F10" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G10" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="H10" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I10" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J10" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="K10" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="M10" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="P10" s="41" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="O2" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P2" s="40" t="inlineStr">
+    </row>
+    <row r="11">
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="E11" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="F11" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G11" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="H11" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J11" s="49" t="inlineStr">
         <is>
           <t>WS B - 2</t>
         </is>
       </c>
-      <c r="Q2" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="R2" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="S2" s="41" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="T2" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="U2" s="41" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="V2" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="W2" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="X2" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="Y2" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="Z2" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AA2" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="AB2" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AC2" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="AD2" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="AE2" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="33" t="inlineStr">
+      <c r="K11" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="M11" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="P11" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C3" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D3" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E3" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F3" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="G3" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="H3" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="I3" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J3" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="K3" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L3" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M3" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N3" s="39" t="inlineStr">
+      <c r="E12" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="G12" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="I12" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J12" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="K12" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="M12" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="P12" s="41" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="O3" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P3" s="40" t="inlineStr">
+    </row>
+    <row r="13">
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E13" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="G13" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="I13" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J13" s="49" t="inlineStr">
         <is>
           <t>WS B - 2</t>
         </is>
       </c>
-      <c r="Q3" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="R3" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="S3" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="T3" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="U3" s="41" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="V3" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="W3" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="X3" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="Y3" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="Z3" s="40" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="AB3" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C4" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D4" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F4" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="G4" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="H4" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I4" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J4" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="K4" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L4" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M4" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N4" s="39" t="inlineStr">
+      <c r="K13" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="M13" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="P13" s="41" t="inlineStr">
         <is>
           <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="O4" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P4" s="40" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="Q4" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
-        </is>
-      </c>
-      <c r="R4" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="S4" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="T4" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="U4" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="V4" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="W4" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="X4" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="Y4" s="42" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="Z4" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
-        </is>
-      </c>
-      <c r="AB4" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C5" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D5" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E5" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F5" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="G5" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="H5" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I5" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J5" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="K5" s="36" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L5" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M5" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N5" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="O5" s="35" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="P5" s="40" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="R5" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="S5" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="T5" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="U5" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="V5" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="W5" s="41" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="X5" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="Y5" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C6" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D6" s="34" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E6" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="G6" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H6" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I6" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J6" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K6" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="L6" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M6" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="O6" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="P6" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="R6" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S6" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="T6" s="40" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="U6" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="V6" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="W6" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="X6" s="50" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="Y6" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D7" s="40" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="E7" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F7" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="G7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H7" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I7" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J7" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="L7" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M7" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="O7" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="P7" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="R7" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S7" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="T7" s="40" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="U7" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="V7" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="W7" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D8" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E8" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F8" s="38" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="G8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H8" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I8" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J8" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K8" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="L8" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M8" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="O8" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="P8" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="R8" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S8" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="U8" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D9" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E9" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F9" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="G9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H9" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I9" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J9" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K9" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="L9" s="39" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M9" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="O9" s="46" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="P9" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="R9" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S9" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="U9" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C10" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="D10" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E10" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="F10" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="G10" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H10" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I10" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J10" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K10" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="M10" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="O10" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="R10" s="50" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C11" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="D11" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E11" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="F11" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="G11" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H11" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="I11" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J11" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K11" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="M11" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="O11" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="R11" s="50" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="E12" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="F12" s="43" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="G12" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H12" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="I12" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J12" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K12" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="M12" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="O12" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="E13" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="G13" s="45" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H13" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="I13" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J13" s="48" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K13" s="49" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="M13" s="51" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="O13" s="47" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add checking for umpire matches
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -21449,7 +21449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="27.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -22193,6 +22193,169 @@
         </is>
       </c>
       <c r="C67" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (XD B, MD C, XD C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Log entry at 2025-10-15 16:11:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>⚠️ Linnea Vainula</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>plays WD V, so cannot play WD A</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>⚠️ Linnea Vainula</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (WD A, WD V, XD V)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>⚠️ Viivi Brandt</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>plays WD V, so cannot play WD A</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>⚠️ Viivi Brandt</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (WD A, WD V, XD V)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>⚠️ Elina Heikkilä</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (WD A, XD B, WD B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>⚠️ Tuomas Järvinen</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>participates in 4 events (XD C, XD B, MD C, MD B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>⚠️ Tuomas Järvinen</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>plays 4 doubles classes (XD C, XD B, MD C, MD B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>⚠️ Alexander Lindholm</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (MD A, XD B, MD B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>⚠️ Otso Pennanen</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>participates in 4 events (XD B, MD C, MS C, XD C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>⚠️ Otso Pennanen</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (XD B, MD C, XD C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>⚠️ Xin Zhang</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>participates in 4 events (WD C, XD B, XD C, WS C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>⚠️ Xin Zhang</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>plays 3 doubles classes (WD C, XD B, XD C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>⚠️ Hanchen Wang</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
         <is>
           <t>plays 3 doubles classes (XD B, MD C, XD C)</t>
         </is>
@@ -22271,7 +22434,7 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>MD V (10), XD A (1), XD V (2)</t>
+          <t>MD V (10), XD V (2), XD A (1)</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
@@ -22300,7 +22463,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>XD A (4), WD V (8), XD V (3), WD A (1)</t>
+          <t>WD V (8), XD V (3), XD A (4), WD A (1)</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
@@ -22329,7 +22492,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>MS V (7), XD A (4), XD V (8), MS A (4)</t>
+          <t>XD V (8), MS A (4), XD A (4), MS V (7)</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
@@ -22358,7 +22521,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>XD A (3), WS V (9), XD V (10), WS A (1)</t>
+          <t>XD V (10), WS V (9), XD A (3), WS A (1)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
@@ -22385,7 +22548,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>WD V (12), WS A (2), MD V (8), WD A (2), WS V (4), MD A (4), MS V (4)</t>
+          <t>WD V (12), WS V (4), MD A (4), MS V (4), MD V (8), WS A (2), WD A (2)</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
@@ -22414,7 +22577,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>MD A (13), XD B (2), MD B (6), XD A (6), MS B (1)</t>
+          <t>MD A (13), MD B (6), XD B (2), XD A (6), MS B (1)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
@@ -22445,7 +22608,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>XD A (2), WD A (3), XD B (1), WD B (1), WD V (1), XD V (1)</t>
+          <t>XD A (2), WD V (1), XD V (1), WD A (3), XD B (1), WD B (1)</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
@@ -22472,7 +22635,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>XD V (2), XD A (1), MS A (1), MD B (1)</t>
+          <t>XD V (2), MD B (1), MS A (1), XD A (1)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
@@ -22499,7 +22662,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>XD A (4), WS A (6), XD B (2), WD B (1), WD V (2), XD V (2)</t>
+          <t>XD B (2), WD B (1), WD V (2), XD V (2), WS A (6), XD A (4)</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -22526,7 +22689,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>WD A (6), MD A (7), MD V (3), WS A (3), MD B (1), WS V (3), MS A (5), WD B (1), WD V (4), WS B (1), MS V (1), XD B (1), MS B (1)</t>
+          <t>WD V (4), MS B (1), WD A (6), MD A (7), WS A (3), MD V (3), MS V (1), MS A (5), WS B (1), WD B (1), MD B (1), WS V (3), XD B (1)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
@@ -22555,7 +22718,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>XD B (4), MD A (3), MD B (8), MS A (2), MS C (2), XD A (1)</t>
+          <t>XD A (1), MD B (8), MS C (2), MD A (3), XD B (4), MS A (2)</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
@@ -22586,7 +22749,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>WD A (2), WD B (3), XD C (2), XD A (2), WD C (1), XD B (1), WD V (1)</t>
+          <t>WD A (2), XD A (2), WD B (3), XD C (2), XD B (1), WD C (1), WD V (1)</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
@@ -22615,7 +22778,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>MS B (14), XD B (7), MS A (6), XD A (1), MD C (5), XD C (4), MS C (5), MD A (3)</t>
+          <t>MS C (5), MS A (6), MS B (14), XD B (7), XD C (4), MD C (5), MD A (3), XD A (1)</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
@@ -22646,7 +22809,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>XD B (5), WD A (1), XD C (1), WS B (2), WS A (1), WS C (1)</t>
+          <t>XD B (5), WD A (1), XD C (1), WS B (2), WS C (1), WS A (1)</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
@@ -22671,7 +22834,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>MS B (7), MD B (6), WD B (8), MS A (3), MD A (7), WD A (2), WS C (3), WD C (2), XD A (1), WS B (2), WS A (2), MS C (1), MD C (1), XD C (1)</t>
+          <t>WD B (8), WS A (2), MS A (3), MD B (6), MS B (7), MD A (7), WS B (2), WD C (2), WS C (3), MD C (1), MS C (1), XD C (1), WD A (2), XD A (1)</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
@@ -22700,7 +22863,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>MD C (14), XD C (6), MD B (3), MS B (1)</t>
+          <t>MD B (3), MD C (14), XD C (6), MS B (1)</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
@@ -22733,7 +22896,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>WD C (7), XD C (5), XD B (3), WS B (1)</t>
+          <t>WD C (7), XD B (3), XD C (5), WS B (1)</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
@@ -22762,7 +22925,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>XD C (5), MS C (11), XD B (2), MD B (4)</t>
+          <t>MS C (11), XD C (5), XD B (2), MD B (4)</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
@@ -22791,7 +22954,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>XD C (7), WS C (7), XD B (3), WS B (1)</t>
+          <t>XD C (7), XD B (3), WS C (7), WS B (1)</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
@@ -22818,7 +22981,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>MS C (5), WS C (3), WD C (3), MD C (5), MD B (1), WD B (2), WS B (2)</t>
+          <t>MD C (5), MS C (5), WD B (2), WD C (3), WS B (2), WS C (3), MD B (1)</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
@@ -22848,691 +23011,721 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AM13"/>
+  <dimension ref="B2:AQ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="C2" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C2" s="34" t="inlineStr">
+      <c r="D2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="E2" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="F2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="G2" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="H2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="I2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="K2" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="L2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="M2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="N2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="O2" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="P2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="Q2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R2" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="S2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="U2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AA2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AB2" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AC2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AD2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AE2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AF2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AG2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AH2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
+        </is>
+      </c>
+      <c r="AI2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AK2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="AL2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+      <c r="AM2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+      <c r="AN2" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AO2" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+      <c r="AQ2" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="C3" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="D2" s="35" t="inlineStr">
+      <c r="D3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="E3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="F3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="G3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="H3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="I3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="K3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="L3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="M3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="N3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="O3" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="P3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="Q3" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R3" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="S3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="U3" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AA3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AB3" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AC3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AD3" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AE3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AF3" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AG3" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="AH3" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AI3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ3" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AK3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="AM3" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AN3" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="E2" s="34" t="inlineStr">
+      <c r="C4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="E4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="F4" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="G4" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F2" s="36" t="inlineStr">
+      <c r="H4" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="I4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J4" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="K4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="L4" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="M4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="N4" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="O4" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="P4" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="Q4" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R4" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="S4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="U4" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AA4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AB4" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AC4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AD4" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AE4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AF4" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AG4" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="AI4" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AK4" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AM4" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="G2" s="37" t="inlineStr">
+      <c r="E5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="F5" s="37" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="H2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="I2" s="39" t="inlineStr">
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="H5" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="I5" s="39" t="inlineStr">
         <is>
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="J2" s="40" t="inlineStr">
+      <c r="J5" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="K5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="L5" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="M5" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="N5" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O5" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="P5" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="Q5" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R5" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="S5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="U5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AA5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AB5" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AC5" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AE5" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AI5" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AK5" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="H6" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="I6" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J6" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K6" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="L6" s="40" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="K2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L2" s="41" t="inlineStr">
+      <c r="M6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="N6" s="41" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="M2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N2" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="P2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q2" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="R2" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S2" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="AA2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AB2" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AD2" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AE2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AF2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AG2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="AH2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AI2" s="45" t="inlineStr">
+      <c r="O6" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="AA6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AB6" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AC6" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+      <c r="AE6" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AI6" s="45" t="inlineStr">
         <is>
           <t>MD A - 2</t>
         </is>
       </c>
-      <c r="AJ2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="AK2" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AL2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AM2" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E3" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="G3" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="I3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J3" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="K3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L3" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="P3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q3" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="R3" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S3" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="AA3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AB3" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AD3" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AE3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AF3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AG3" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="AH3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
-        </is>
-      </c>
-      <c r="AI3" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AK3" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="AL3" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C4" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D4" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F4" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="G4" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="I4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J4" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="K4" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L4" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M4" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="P4" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q4" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="R4" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="S4" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="AA4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AB4" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AC4" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AD4" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="AE4" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AF4" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AG4" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-      <c r="AH4" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AI4" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ4" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AK4" s="52" t="inlineStr">
+      <c r="AK6" s="52" t="inlineStr">
         <is>
           <t>XD C - 3</t>
-        </is>
-      </c>
-      <c r="AL4" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C5" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D5" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F5" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="G5" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="I5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="K5" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="L5" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M5" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="N5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="P5" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="Q5" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="R5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AB5" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AC5" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AE5" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AF5" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AI5" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ5" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D6" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="E6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="F6" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="G6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H6" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="I6" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="K6" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="L6" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="M6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="N6" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="P6" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AA6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AB6" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AC6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AE6" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AF6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="AI6" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
         </is>
       </c>
     </row>
@@ -23542,69 +23735,64 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D7" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="G7" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F7" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="G7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H7" s="42" t="inlineStr">
+      <c r="H7" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="I7" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J7" s="42" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="I7" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J7" s="40" t="inlineStr">
+      <c r="K7" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="L7" s="40" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="K7" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="L7" s="41" t="inlineStr">
+      <c r="M7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="N7" s="41" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="M7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="N7" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="P7" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
+      <c r="O7" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
         </is>
       </c>
       <c r="AA7" s="37" t="inlineStr">
@@ -23617,24 +23805,14 @@
           <t>MD B - 4</t>
         </is>
       </c>
-      <c r="AC7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
       <c r="AE7" s="50" t="inlineStr">
         <is>
           <t>WD C - 2</t>
         </is>
       </c>
-      <c r="AF7" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AI7" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
+      <c r="AI7" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
         </is>
       </c>
     </row>
@@ -23649,59 +23827,59 @@
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="D8" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E8" s="34" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F8" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="G8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H8" s="42" t="inlineStr">
+      <c r="H8" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="I8" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J8" s="42" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="I8" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J8" s="40" t="inlineStr">
+      <c r="K8" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="L8" s="40" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="K8" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="L8" s="41" t="inlineStr">
+      <c r="M8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="N8" s="41" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="M8" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="P8" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
+      <c r="O8" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
         </is>
       </c>
       <c r="AA8" s="53" t="inlineStr">
@@ -23709,14 +23887,14 @@
           <t>WS C - 3</t>
         </is>
       </c>
-      <c r="AC8" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
-        </is>
-      </c>
-      <c r="AF8" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
+      <c r="AE8" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AI8" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
         </is>
       </c>
     </row>
@@ -23731,64 +23909,69 @@
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E9" s="34" t="inlineStr">
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="H9" s="40" t="inlineStr">
         <is>
           <t>MS B - 1</t>
         </is>
       </c>
-      <c r="G9" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="H9" s="42" t="inlineStr">
+      <c r="I9" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="J9" s="42" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="I9" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="K9" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="L9" s="40" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="K9" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="L9" s="41" t="inlineStr">
+      <c r="M9" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="N9" s="41" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="M9" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="P9" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
+      <c r="O9" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
         </is>
       </c>
       <c r="AA9" s="53" t="inlineStr">
         <is>
           <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AI9" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
         </is>
       </c>
     </row>
@@ -23798,24 +23981,19 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C10" s="53" t="inlineStr">
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D10" s="53" t="inlineStr">
         <is>
           <t>WS C - 1</t>
         </is>
       </c>
-      <c r="D10" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E10" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="F10" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
         </is>
       </c>
       <c r="G10" s="53" t="inlineStr">
@@ -23823,34 +24001,34 @@
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="H10" s="42" t="inlineStr">
+      <c r="H10" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="I10" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="J10" s="42" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="I10" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J10" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="K10" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="M10" s="46" t="inlineStr">
+      <c r="K10" s="46" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="P10" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
+      <c r="L10" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="N10" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
         </is>
       </c>
     </row>
@@ -23860,24 +24038,19 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="C11" s="53" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D11" s="53" t="inlineStr">
         <is>
           <t>WS C - 1</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="E11" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="F11" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
         </is>
       </c>
       <c r="G11" s="53" t="inlineStr">
@@ -23885,34 +24058,34 @@
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="H11" s="42" t="inlineStr">
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="I11" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="J11" s="42" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="I11" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J11" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="K11" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="M11" s="46" t="inlineStr">
+      <c r="K11" s="46" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="P11" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
+      <c r="L11" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="N11" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
         </is>
       </c>
     </row>
@@ -23922,14 +24095,9 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="E12" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="F12" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
         </is>
       </c>
       <c r="G12" s="53" t="inlineStr">
@@ -23937,29 +24105,29 @@
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="I12" s="46" t="inlineStr">
+      <c r="H12" s="46" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="J12" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="K12" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="M12" s="46" t="inlineStr">
+      <c r="J12" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K12" s="46" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="P12" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
+      <c r="L12" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="N12" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
         </is>
       </c>
     </row>
@@ -23969,9 +24137,9 @@
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="E13" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
         </is>
       </c>
       <c r="G13" s="53" t="inlineStr">
@@ -23979,29 +24147,24 @@
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="I13" s="46" t="inlineStr">
+      <c r="H13" s="46" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="J13" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="K13" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="M13" s="46" t="inlineStr">
+      <c r="J13" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="K13" s="46" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="P13" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
+      <c r="L13" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
lots of stuff and solver using chuffed now
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -23011,1160 +23011,1160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AQ13"/>
+  <dimension ref="B2:AR13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="35" t="inlineStr">
+      <c r="B2" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="D2" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="E2" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="F2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="G2" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="H2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="J2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="L2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="M2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="O2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="P2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="S2" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T2" s="35" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="C2" s="34" t="inlineStr">
+      <c r="U2" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="V2" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="X2" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="D2" s="36" t="inlineStr">
+      <c r="Y2" s="36" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="E2" s="49" t="inlineStr">
+      <c r="Z2" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AA2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AB2" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AC2" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AD2" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AE2" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AF2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="AG2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AH2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AI2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AJ2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AK2" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AL2" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AM2" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AN2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AO2" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AP2" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="AQ2" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AR2" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="D3" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="F3" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="G3" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="H3" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="J3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="L3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="M3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="O3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="P3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="S3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="U3" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="V3" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="X3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="Y3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="Z3" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AA3" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AB3" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AC3" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AD3" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AE3" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AF3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="AG3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AH3" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AI3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AJ3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AK3" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="AL3" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AM3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AN3" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AO3" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AP3" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AQ3" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AR3" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="J4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="L4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="O4" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="P4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="S4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T4" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="V4" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W4" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="X4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="Y4" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="Z4" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AA4" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AC4" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AD4" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AE4" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AF4" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AG4" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AH4" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AI4" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AJ4" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AL4" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AM4" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AN4" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="AO4" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AP4" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AQ4" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AR4" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="H5" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="J5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="L5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="O5" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="P5" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="S5" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T5" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="V5" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W5" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="X5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="Y5" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="Z5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AA5" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AC5" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AD5" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AE5" s="48" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AF5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AG5" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AH5" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AI5" s="47" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AJ5" s="36" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AL5" s="38" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AM5" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AN5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AO5" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AP5" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AR5" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="P6" s="39" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="S6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T6" s="35" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="V6" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="Y6" s="49" t="inlineStr">
         <is>
           <t>WS B - 1</t>
         </is>
       </c>
-      <c r="F2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="G2" s="34" t="inlineStr">
+      <c r="Z6" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="AA6" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AC6" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AE6" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AF6" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AG6" s="51" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AH6" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AI6" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="H2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="I2" s="39" t="inlineStr">
+      <c r="AJ6" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AL6" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+      <c r="AM6" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="AN6" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AO6" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AP6" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="F7" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="L7" s="42" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="P7" s="39" t="inlineStr">
         <is>
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="J2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="K2" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="L2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="M2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="N2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="O2" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="P2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="Q2" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R2" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S2" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="U2" s="40" t="inlineStr">
+      <c r="S7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="V7" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X7" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="Z7" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="AA7" s="46" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AC7" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AE7" s="45" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AF7" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AH7" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AI7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ7" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AM7" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="AN7" s="40" t="inlineStr">
         <is>
           <t>MS B - 3</t>
         </is>
       </c>
-      <c r="AA2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AB2" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AD2" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AE2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AF2" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="AG2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="AH2" s="42" t="inlineStr">
+      <c r="AO7" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AP7" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="S8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="V8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="W8" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X8" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="AF8" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AH8" s="42" t="inlineStr">
         <is>
           <t>MD B - 5</t>
         </is>
       </c>
-      <c r="AI2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AJ2" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AK2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AL2" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-      <c r="AM2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="AN2" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AO2" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="AQ2" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="C3" s="34" t="inlineStr">
+      <c r="AI8" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ8" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AM8" s="43" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="AN8" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AO8" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AP8" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="S9" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="V9" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="W9" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="D3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="E3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="F3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="G3" s="34" t="inlineStr">
+      <c r="X9" s="44" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="AF9" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AI9" s="34" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="H3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="I3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="K3" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="L3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="M3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="N3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="O3" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="P3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="Q3" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R3" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="U3" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AB3" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AD3" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AE3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AF3" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AG3" s="46" t="inlineStr">
+      <c r="AJ9" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AN9" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="S10" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="V10" s="50" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="W10" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X10" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AF10" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AI10" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ10" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AN10" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="S11" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="W11" s="34" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X11" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AF11" s="40" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AI11" s="46" t="inlineStr">
         <is>
           <t>MD C - 4</t>
         </is>
       </c>
-      <c r="AH3" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AI3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AJ3" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AK3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AM3" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AN3" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="C4" s="34" t="inlineStr">
+      <c r="AJ11" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AN11" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="S12" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="W12" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="D4" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="E4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="F4" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="H4" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="I4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J4" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="K4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="L4" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="M4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="N4" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="O4" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="P4" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="Q4" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R4" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="U4" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AB4" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AC4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AD4" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="AE4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AF4" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AG4" s="50" t="inlineStr">
+      <c r="X12" s="37" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AF12" s="52" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AI12" s="50" t="inlineStr">
         <is>
           <t>WD C - 3</t>
         </is>
       </c>
-      <c r="AI4" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AK4" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="AM4" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="AJ12" s="49" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AN12" s="53" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="W13" s="34" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="D5" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="E5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="F5" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="H5" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="I5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J5" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="K5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="L5" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="M5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="N5" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="O5" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="P5" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="Q5" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R5" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="S5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="U5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AB5" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AC5" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="AE5" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AI5" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AK5" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="C6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="D6" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="E6" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="F6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="H6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="I6" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J6" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K6" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="L6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="M6" s="37" t="inlineStr">
+      <c r="X13" s="37" t="inlineStr">
         <is>
           <t>MS C - 3</t>
         </is>
       </c>
-      <c r="N6" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="O6" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="AA6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AB6" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AC6" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
-        </is>
-      </c>
-      <c r="AE6" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AI6" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AK6" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="F7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="H7" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="I7" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="J7" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K7" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="L7" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="M7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="N7" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="O7" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="AA7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AB7" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AE7" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AI7" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D8" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="F8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G8" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="H8" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="I8" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J8" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K8" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="L8" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="M8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="N8" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="O8" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="AA8" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="AE8" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AI8" s="52" t="inlineStr">
+      <c r="AF13" s="52" t="inlineStr">
         <is>
           <t>XD C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D9" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G9" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="H9" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="I9" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J9" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K9" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="L9" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="M9" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="N9" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="O9" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="AA9" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="AI9" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C10" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D10" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G10" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="H10" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="I10" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="J10" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K10" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="L10" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="N10" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="D11" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="G11" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="H11" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="I11" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="J11" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K11" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="L11" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="N11" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C12" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="G12" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="H12" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J12" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K12" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="L12" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="N12" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="G13" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="H13" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="J13" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="K13" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="L13" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Umpire matches are taken into account now
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Entries HBC Premier Elite 2024" sheetId="1" state="visible" r:id="rId1"/>
@@ -60,7 +60,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="44">
+  <fills count="45">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +70,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -141,12 +147,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFD54F"/>
-        <bgColor rgb="FFFFD54F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF66BB6A"/>
         <bgColor rgb="FF66BB6A"/>
       </patternFill>
@@ -159,20 +159,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF64B5F6"/>
+        <bgColor rgb="FF64B5F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFEC407A"/>
         <bgColor rgb="FFEC407A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF64B5F6"/>
-        <bgColor rgb="FF64B5F6"/>
+        <fgColor rgb="FFFFD54F"/>
+        <bgColor rgb="FFFFD54F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF06292"/>
-        <bgColor rgb="FFF06292"/>
+        <fgColor rgb="FFC8E6C9"/>
+        <bgColor rgb="FFC8E6C9"/>
       </patternFill>
     </fill>
     <fill>
@@ -189,13 +195,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC8E6C9"/>
-        <bgColor rgb="FFC8E6C9"/>
+        <fgColor rgb="FFF06292"/>
+        <bgColor rgb="FFF06292"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -237,8 +243,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCA28"/>
-        <bgColor rgb="00FFCA28"/>
+        <fgColor rgb="0066BB6A"/>
+        <bgColor rgb="0066BB6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE0E0"/>
+        <bgColor rgb="00FDE0E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -249,38 +261,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BBDEFB"/>
-        <bgColor rgb="00BBDEFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDE0E0"/>
-        <bgColor rgb="00FDE0E0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0090CAF9"/>
-        <bgColor rgb="0090CAF9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0066BB6A"/>
-        <bgColor rgb="0066BB6A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFE082"/>
         <bgColor rgb="00FFE082"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0064B5F6"/>
-        <bgColor rgb="0064B5F6"/>
+        <fgColor rgb="00FFD54F"/>
+        <bgColor rgb="00FFD54F"/>
       </patternFill>
     </fill>
     <fill>
@@ -291,14 +279,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD54F"/>
-        <bgColor rgb="00FFD54F"/>
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
-        <bgColor rgb="00C8E6C9"/>
+        <fgColor rgb="0090CAF9"/>
+        <bgColor rgb="0090CAF9"/>
       </patternFill>
     </fill>
     <fill>
@@ -311,6 +299,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="0081C784"/>
         <bgColor rgb="0081C784"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCA28"/>
+        <bgColor rgb="00FFCA28"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0064B5F6"/>
+        <bgColor rgb="0064B5F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -341,7 +347,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -369,47 +375,48 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="43" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14064,7 +14071,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="AO25" s="33" t="inlineStr">
+      <c r="AO25" s="13" t="inlineStr">
         <is>
           <t>En klass måste ha min 60 min mällan sina rundor</t>
         </is>
@@ -14088,7 +14095,7 @@
           <t>XD B</t>
         </is>
       </c>
-      <c r="AO26" s="33" t="inlineStr">
+      <c r="AO26" s="13" t="inlineStr">
         <is>
           <t>Alla matcher i en runda måste sättas in i max två efterföljande (jämna) tidsslots</t>
         </is>
@@ -14118,7 +14125,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="AO28" s="33" t="inlineStr">
+      <c r="AO28" s="13" t="inlineStr">
         <is>
           <t>En tidsslot kan ha max 10 matcher</t>
         </is>
@@ -14224,7 +14231,7 @@
       <c r="AH29" s="3" t="n">
         <v>0.8958333333333334</v>
       </c>
-      <c r="AO29" s="2" t="inlineStr">
+      <c r="AO29" s="34" t="inlineStr">
         <is>
           <t>Det får inte spelas mer än 4 domarmatcher på en tidsslot</t>
         </is>
@@ -14394,7 +14401,7 @@
           <t>MD B</t>
         </is>
       </c>
-      <c r="AO30" s="2" t="inlineStr">
+      <c r="AO30" s="34" t="inlineStr">
         <is>
           <t>Domarmatcher måste ha min 45 min mällan sig</t>
         </is>
@@ -14724,7 +14731,7 @@
           <t>MD B</t>
         </is>
       </c>
-      <c r="AO32" s="33" t="inlineStr">
+      <c r="AO32" s="13" t="inlineStr">
         <is>
           <t>Innom en nivå måste alla rundor i kolliderande klasser spelas med minst 1 tom tidsslots mällanrum</t>
         </is>
@@ -14879,7 +14886,7 @@
           <t>MD B</t>
         </is>
       </c>
-      <c r="AO33" s="33" t="inlineStr">
+      <c r="AO33" s="13" t="inlineStr">
         <is>
           <t>Rundor i kolliderande klasser som inte hör till samma nivå får inte spelas på samma tidsslot</t>
         </is>
@@ -15164,7 +15171,7 @@
           <t>MD A</t>
         </is>
       </c>
-      <c r="AO35" s="33" t="inlineStr">
+      <c r="AO35" s="13" t="inlineStr">
         <is>
           <t>Alla matcher ska spelas exakt en gång</t>
         </is>
@@ -15294,7 +15301,7 @@
           <t>MD A</t>
         </is>
       </c>
-      <c r="AO36" s="33" t="inlineStr">
+      <c r="AO36" s="13" t="inlineStr">
         <is>
           <t>Alla icke domarmatcher får bara spelas i timeslots som är prick och halv</t>
         </is>
@@ -18296,8 +18303,8 @@
     <col width="29.6640625" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="20.6640625" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
     <col width="34.33203125" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
-    <col width="8.83203125" customWidth="1" style="7" min="4" max="12"/>
-    <col width="8.83203125" customWidth="1" style="7" min="13" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="7" min="4" max="13"/>
+    <col width="8.83203125" customWidth="1" style="7" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" thickBot="1">
@@ -23015,1156 +23022,1156 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="52" t="inlineStr">
+      <c r="B2" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="C2" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="E2" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="F2" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="G2" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I2" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="K2" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="L2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="M2" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="N2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="O2" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="P2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="R2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="S2" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="U2" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="V2" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="W2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="X2" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="Z2" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AA2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AB2" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AC2" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AD2" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AE2" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AG2" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+      <c r="AH2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="AI2" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AK2" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AL2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="AM2" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AN2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AO2" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AP2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AQ2" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AR2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="F3" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="G3" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I3" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="K3" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="L3" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="M3" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="P3" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="R3" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="S3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T3" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="U3" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="W3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X3" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y3" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="Z3" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AA3" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AB3" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AC3" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AD3" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AE3" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF3" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AH3" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AI3" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ3" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AK3" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AL3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="AM3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AN3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AO3" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AP3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AQ3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AR3" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="E4" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="F4" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="G4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="K4" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="L4" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="M4" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="P4" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="R4" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="S4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T4" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="U4" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="W4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X4" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y4" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="Z4" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AA4" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AB4" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AC4" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AD4" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AE4" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AH4" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AI4" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AJ4" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AK4" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AL4" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AM4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AN4" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AO4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AP4" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+      <c r="AR4" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="F5" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="G5" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I5" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="K5" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="L5" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="M5" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="R5" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="S5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T5" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="U5" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="W5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X5" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y5" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="Z5" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AA5" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AB5" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AC5" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="AD5" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AE5" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF5" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="AH5" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AI5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AJ5" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AK5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AL5" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AM5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AN5" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AO5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AP5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AR5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="G6" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I6" s="53" t="inlineStr">
         <is>
           <t>XD C - 1</t>
         </is>
       </c>
-      <c r="D2" s="46" t="inlineStr">
+      <c r="K6" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="M6" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="P6" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="R6" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="S6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T6" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="U6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="W6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y6" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AA6" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AC6" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AD6" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AE6" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
+        </is>
+      </c>
+      <c r="AF6" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="AH6" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AI6" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AK6" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AL6" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AM6" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AN6" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AP6" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AR6" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="F7" s="49" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="E2" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F2" s="41" t="inlineStr">
+      <c r="G7" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I7" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="M7" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="S7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T7" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="U7" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X7" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y7" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AA7" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AC7" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AD7" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AH7" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AI7" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AK7" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AL7" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AM7" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AN7" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AP7" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="G2" s="46" t="inlineStr">
+      <c r="I8" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="M8" s="49" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="H2" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="J2" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="L2" s="42" t="inlineStr">
+      <c r="S8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="T8" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="M2" s="42" t="inlineStr">
+      <c r="U8" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X8" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y8" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AH8" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AI8" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="AK8" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AM8" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AN8" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AP8" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="I9" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="T9" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="O2" s="42" t="inlineStr">
+      <c r="U9" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X9" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="Y9" s="45" t="inlineStr">
         <is>
           <t>MD B - 3</t>
         </is>
       </c>
-      <c r="P2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="S2" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="T2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="U2" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="V2" s="37" t="inlineStr">
+      <c r="AK9" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AM9" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AN9" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="T10" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="U10" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X10" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="W2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="X2" s="34" t="inlineStr">
+      <c r="AK10" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AN10" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="T11" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="U11" s="35" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="Y2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="Z2" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AA2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AB2" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AC2" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AD2" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AE2" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AF2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="AG2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AH2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AI2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AJ2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AK2" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="AL2" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AM2" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AN2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AO2" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AP2" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AQ2" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AR2" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D3" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F3" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="G3" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="H3" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="J3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="L3" s="42" t="inlineStr">
+      <c r="X11" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AK11" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="T12" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="M3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="O3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="P3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="S3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="T3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="U3" s="37" t="inlineStr">
+      <c r="U12" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X12" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="V3" s="37" t="inlineStr">
+      <c r="AK12" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="U13" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="X13" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="W3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="X3" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="Y3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="Z3" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AA3" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AB3" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AC3" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="AD3" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AE3" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AF3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="AG3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AH3" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AI3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AJ3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AK3" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
-        </is>
-      </c>
-      <c r="AL3" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AM3" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AN3" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AO3" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AP3" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AQ3" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="AR3" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D4" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F4" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="G4" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="H4" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="J4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="L4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="O4" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="P4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="S4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="T4" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="V4" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="W4" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="X4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="Y4" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="Z4" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AA4" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AC4" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AD4" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AE4" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AF4" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AG4" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AH4" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AI4" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AJ4" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL4" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AM4" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AN4" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AO4" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AP4" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AQ4" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="AR4" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D5" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F5" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="G5" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="H5" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="J5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="L5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="O5" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="P5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="S5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="T5" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="V5" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="W5" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="X5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="Y5" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="Z5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AA5" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AC5" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AD5" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AE5" s="48" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AF5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AG5" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AH5" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AI5" s="47" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AJ5" s="36" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL5" s="38" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AM5" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AN5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AO5" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AP5" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AR5" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="D6" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F6" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="L6" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P6" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="S6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T6" s="35" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="V6" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="W6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="Y6" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="Z6" s="53" t="inlineStr">
+      <c r="AK13" s="51" t="inlineStr">
         <is>
           <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="AA6" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AC6" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AE6" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AF6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AG6" s="51" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AH6" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AI6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ6" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AL6" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-      <c r="AM6" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AN6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AO6" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AP6" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="F7" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="L7" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P7" s="39" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="S7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="V7" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="W7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X7" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Z7" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="AA7" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AC7" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AE7" s="45" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AF7" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AH7" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AI7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ7" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AM7" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AN7" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AO7" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AP7" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="F8" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="S8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="V8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="W8" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X8" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="AF8" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AH8" s="42" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
-        </is>
-      </c>
-      <c r="AI8" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ8" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AM8" s="43" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AN8" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AO8" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="AP8" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="F9" s="41" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="S9" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="V9" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="W9" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X9" s="44" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="AF9" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AI9" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ9" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AN9" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="S10" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="V10" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="W10" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X10" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AF10" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AI10" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ10" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AN10" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="S11" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="W11" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X11" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AF11" s="40" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AI11" s="46" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="AJ11" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AN11" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="S12" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="W12" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X12" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AF12" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="AI12" s="50" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-      <c r="AJ12" s="49" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AN12" s="53" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="W13" s="34" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X13" s="37" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AF13" s="52" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
försök med 15 min intervaller
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024 copy.xlsx
+++ b/Entries HBC Premier Elite 2024 copy.xlsx
@@ -23018,7 +23018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR13"/>
+  <dimension ref="B2:BA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -23032,526 +23032,536 @@
           <t>XD B - 1</t>
         </is>
       </c>
+      <c r="D2" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
       <c r="E2" s="40" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="F2" s="49" t="inlineStr">
+      <c r="G2" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="I2" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="J2" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="K2" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="S2" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="U2" s="49" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="G2" s="37" t="inlineStr">
+      <c r="V2" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="X2" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="Z2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="AB2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="AC2" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="AD2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="AE2" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="AH2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AI2" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ2" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AK2" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AL2" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AM2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AN2" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="AO2" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AP2" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AQ2" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AR2" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+      <c r="AS2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="AT2" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AU2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AV2" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AW2" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AX2" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AY2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AZ2" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="BA2" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="D3" s="37" t="inlineStr">
         <is>
           <t>XD A - 1</t>
         </is>
       </c>
-      <c r="I2" s="37" t="inlineStr">
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="G3" s="37" t="inlineStr">
         <is>
           <t>XD A - 2</t>
         </is>
       </c>
-      <c r="K2" s="42" t="inlineStr">
+      <c r="I3" s="42" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="L2" s="36" t="inlineStr">
+      <c r="J3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="K3" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="S3" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="U3" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="V3" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="X3" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="Z3" s="36" t="inlineStr">
         <is>
           <t>XD V - 1</t>
         </is>
       </c>
-      <c r="M2" s="46" t="inlineStr">
+      <c r="AB3" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="AC3" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="AD3" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="AE3" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF3" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="AH3" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AI3" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ3" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AK3" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AL3" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AM3" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AN3" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
+        </is>
+      </c>
+      <c r="AO3" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AP3" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AQ3" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AS3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="AT3" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AU3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AV3" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AW3" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AX3" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AY3" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AZ3" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="BA3" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="C4" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="E4" s="40" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="G4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="I4" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="J4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="K4" s="46" t="inlineStr">
         <is>
           <t>WS A - 1</t>
         </is>
       </c>
-      <c r="N2" s="36" t="inlineStr">
+      <c r="S4" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="U4" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="X4" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AB4" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="AC4" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="AD4" s="36" t="inlineStr">
         <is>
           <t>XD V - 2</t>
         </is>
       </c>
-      <c r="O2" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="P2" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="R2" s="38" t="inlineStr">
+      <c r="AE4" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF4" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AH4" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AI4" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ4" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AK4" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AL4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AM4" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AO4" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AP4" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AQ4" s="41" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="AS4" s="38" t="inlineStr">
         <is>
           <t>MS V - 1</t>
         </is>
       </c>
-      <c r="S2" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T2" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="U2" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="V2" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="W2" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="X2" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="Y2" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="Z2" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AA2" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AB2" s="54" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AC2" s="41" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AD2" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AE2" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AF2" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AG2" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-      <c r="AH2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AI2" s="46" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ2" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AK2" s="42" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AL2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AM2" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AN2" s="38" t="inlineStr">
+      <c r="AT4" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AU4" s="38" t="inlineStr">
         <is>
           <t>MS V - 2</t>
         </is>
       </c>
-      <c r="AO2" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AP2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AQ2" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="AR2" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="C3" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="E3" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="F3" s="49" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="G3" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I3" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="K3" s="42" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="L3" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="M3" s="46" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="P3" s="44" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="R3" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="S3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T3" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="U3" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="W3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="X3" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="Y3" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="Z3" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AA3" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AB3" s="54" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AC3" s="41" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AD3" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="AE3" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AF3" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AH3" s="41" t="inlineStr">
+      <c r="AV4" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AW4" s="41" t="inlineStr">
         <is>
           <t>WS V - 2</t>
         </is>
       </c>
-      <c r="AI3" s="46" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AJ3" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AK3" s="42" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="AL3" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AM3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AN3" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AO3" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AP3" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AQ3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="AR3" s="41" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="E4" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="F4" s="49" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="G4" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I4" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="K4" s="42" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="L4" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="M4" s="46" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="P4" s="44" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="R4" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="S4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T4" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="U4" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="W4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="X4" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="Y4" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="Z4" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AA4" s="44" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AB4" s="53" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="AC4" s="41" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AD4" s="49" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AE4" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AF4" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="AH4" s="41" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AI4" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AJ4" s="50" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AK4" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AL4" s="41" t="inlineStr">
+      <c r="AX4" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AY4" s="41" t="inlineStr">
         <is>
           <t>WS V - 3</t>
         </is>
       </c>
-      <c r="AM4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AN4" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AO4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AP4" s="44" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="AR4" s="46" t="inlineStr">
+      <c r="BA4" s="46" t="inlineStr">
         <is>
           <t>WS A - 3</t>
         </is>
@@ -23563,164 +23573,154 @@
           <t>XD B - 1</t>
         </is>
       </c>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="F5" s="49" t="inlineStr">
+      <c r="G5" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="J5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="K5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="S5" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="G5" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I5" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="K5" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="L5" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="M5" s="49" t="inlineStr">
+      <c r="X5" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AB5" s="49" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="P5" s="44" t="inlineStr">
+      <c r="AC5" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="AD5" s="36" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="AE5" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF5" s="44" t="inlineStr">
         <is>
           <t>WD V - 1</t>
         </is>
       </c>
-      <c r="R5" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="S5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T5" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="U5" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="W5" s="47" t="inlineStr">
+      <c r="AH5" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AI5" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AJ5" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AK5" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AL5" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="X5" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="Y5" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="Z5" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AA5" s="44" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AB5" s="53" t="inlineStr">
+      <c r="AM5" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AO5" s="53" t="inlineStr">
         <is>
           <t>XD C - 2</t>
         </is>
       </c>
-      <c r="AC5" s="43" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AD5" s="49" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AE5" s="48" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AF5" s="49" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="AH5" s="41" t="inlineStr">
+      <c r="AP5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="AQ5" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AS5" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="AT5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AU5" s="38" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AV5" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AW5" s="41" t="inlineStr">
         <is>
           <t>WS V - 2</t>
         </is>
       </c>
-      <c r="AI5" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AJ5" s="50" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AK5" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AL5" s="41" t="inlineStr">
+      <c r="AX5" s="52" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AY5" s="41" t="inlineStr">
         <is>
           <t>WS V - 3</t>
         </is>
       </c>
-      <c r="AM5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="AN5" s="38" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AO5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="AP5" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AR5" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
+      <c r="BA5" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
         </is>
       </c>
     </row>
@@ -23730,139 +23730,109 @@
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="F6" s="49" t="inlineStr">
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="J6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="K6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="U6" s="49" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="G6" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I6" s="53" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="K6" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="L6" s="36" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="M6" s="49" t="inlineStr">
+      <c r="AB6" s="49" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="P6" s="44" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="R6" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="S6" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T6" s="45" t="inlineStr">
+      <c r="AD6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AE6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF6" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U6" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="W6" s="47" t="inlineStr">
+      <c r="AH6" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AI6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AK6" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AL6" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="X6" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="Y6" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AA6" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AC6" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AD6" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AE6" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
-        </is>
-      </c>
-      <c r="AF6" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-      <c r="AH6" s="41" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AI6" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AK6" s="39" t="inlineStr">
+      <c r="AM6" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AP6" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AQ6" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AS6" s="44" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+      <c r="AT6" s="39" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="AL6" s="54" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AM6" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="AN6" s="42" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="AP6" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AR6" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
+      <c r="AU6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AW6" s="43" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="AY6" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="BA6" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
         </is>
       </c>
     </row>
@@ -23872,99 +23842,94 @@
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="F7" s="49" t="inlineStr">
+      <c r="D7" s="37" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="U7" s="49" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="G7" s="37" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="I7" s="53" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="M7" s="49" t="inlineStr">
+      <c r="AB7" s="49" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="S7" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T7" s="45" t="inlineStr">
+      <c r="AE7" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF7" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U7" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X7" s="35" t="inlineStr">
+      <c r="AH7" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AI7" s="35" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="Y7" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AA7" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AC7" s="40" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AD7" s="52" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="AH7" s="35" t="inlineStr">
+      <c r="AK7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AL7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AM7" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AP7" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AQ7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AS7" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AT7" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AU7" s="35" t="inlineStr">
         <is>
           <t>MS A - 4</t>
         </is>
       </c>
-      <c r="AI7" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="AK7" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AL7" s="50" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AM7" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="AN7" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AP7" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
+      <c r="AW7" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AY7" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="BA7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
         </is>
       </c>
     </row>
@@ -23974,69 +23939,64 @@
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="I8" s="53" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="M8" s="49" t="inlineStr">
+      <c r="AB8" s="49" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="S8" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="T8" s="45" t="inlineStr">
+      <c r="AE8" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF8" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U8" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X8" s="35" t="inlineStr">
+      <c r="AH8" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AI8" s="35" t="inlineStr">
         <is>
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="Y8" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AH8" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AI8" s="53" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
-        </is>
-      </c>
-      <c r="AK8" s="39" t="inlineStr">
+      <c r="AK8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AQ8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AS8" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AT8" s="39" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="AM8" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="AN8" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AP8" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
+      <c r="AU8" s="42" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AW8" s="54" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AY8" s="46" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
         </is>
       </c>
     </row>
@@ -24046,132 +24006,172 @@
           <t>XD B - 1</t>
         </is>
       </c>
-      <c r="I9" s="53" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="T9" s="45" t="inlineStr">
+      <c r="AE9" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="AF9" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U9" s="35" t="inlineStr">
+      <c r="AI9" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="AK9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AQ9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AS9" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AT9" s="39" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="AU9" s="53" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="AW9" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AY9" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="AE10" s="35" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="X9" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="Y9" s="45" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AK9" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AM9" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="AN9" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="T10" s="45" t="inlineStr">
+      <c r="AF10" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U10" s="35" t="inlineStr">
+      <c r="AK10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AQ10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AS10" s="35" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AT10" s="50" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AW10" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AY10" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="AE11" s="35" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="X10" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AK10" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="AN10" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="T11" s="45" t="inlineStr">
+      <c r="AF11" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U11" s="35" t="inlineStr">
+      <c r="AQ11" s="51" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+      <c r="AS11" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AW11" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AY11" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="AE12" s="35" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="X11" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AK11" s="39" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="T12" s="45" t="inlineStr">
+      <c r="AF12" s="45" t="inlineStr">
         <is>
           <t>MD B - 2</t>
         </is>
       </c>
-      <c r="U12" s="35" t="inlineStr">
+      <c r="AS12" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AW12" s="48" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AY12" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="AE13" s="35" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="X12" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AK12" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="U13" s="35" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="X13" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AK13" s="51" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
+      <c r="AF13" s="45" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="AW13" s="49" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
         </is>
       </c>
     </row>

</xml_diff>